<commit_message>
Program with Datadriven testing
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/TestDatasheet.xlsx
+++ b/src/test/resources/TestData/TestDatasheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91766\IdeaProjects\CucumberBDD1\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEA36735-2D4D-45A0-8FF6-7C258F82BBF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A15BAC0-75C7-4DD2-9B45-DFBD808002DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
   <si>
     <t>Testcase ID</t>
   </si>
@@ -40,6 +40,12 @@
   </si>
   <si>
     <t>admin123</t>
+  </si>
+  <si>
+    <t>TC01</t>
+  </si>
+  <si>
+    <t>TC02</t>
   </si>
 </sst>
 </file>
@@ -375,8 +381,8 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
+      <c r="A2" t="s">
+        <v>5</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -386,8 +392,8 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
+      <c r="A3" t="s">
+        <v>6</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
Getting data from excel
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/TestDatasheet.xlsx
+++ b/src/test/resources/TestData/TestDatasheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91766\IdeaProjects\CucumberBDD1\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A15BAC0-75C7-4DD2-9B45-DFBD808002DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{882081D7-39A7-4896-B020-0AEC28B86A36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t>Testcase ID</t>
   </si>
@@ -46,6 +46,15 @@
   </si>
   <si>
     <t>TC02</t>
+  </si>
+  <si>
+    <t>Adminname</t>
+  </si>
+  <si>
+    <t>Manuel</t>
+  </si>
+  <si>
+    <t>donald</t>
   </si>
 </sst>
 </file>
@@ -363,13 +372,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.21875" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -379,8 +389,11 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -390,8 +403,11 @@
       <c r="C2" t="s">
         <v>4</v>
       </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -400,6 +416,9 @@
       </c>
       <c r="C3" t="s">
         <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>